<commit_message>
updated FOPITY and files for 4.0.5
</commit_message>
<xml_diff>
--- a/InputData/ccs/SoCTaSCbRIC/Share of CCS Transportation and Storage Costs by Recipient ISIC Code.xlsx
+++ b/InputData/ccs/SoCTaSCbRIC/Share of CCS Transportation and Storage Costs by Recipient ISIC Code.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\ccs\SoCTaSCbRIC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\SoCTaSCbRIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1B974E-C82B-4AFB-A807-68E97D691590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FCE592-33B9-486D-B154-CA1C60C6FB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
     <sheet name="SoCTaSCbRIC" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,145 +37,145 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
+    <t>ISIC 97T98</t>
+  </si>
+  <si>
+    <t>ISIC 01T03</t>
+  </si>
+  <si>
+    <t>ISIC 07T08</t>
+  </si>
+  <si>
+    <t>ISIC 09</t>
+  </si>
+  <si>
+    <t>ISIC 10T12</t>
+  </si>
+  <si>
+    <t>ISIC 13T15</t>
+  </si>
+  <si>
+    <t>ISIC 16</t>
+  </si>
+  <si>
+    <t>ISIC 17T18</t>
+  </si>
+  <si>
+    <t>ISIC 19</t>
+  </si>
+  <si>
+    <t>ISIC 22</t>
+  </si>
+  <si>
+    <t>ISIC 25</t>
+  </si>
+  <si>
+    <t>ISIC 26</t>
+  </si>
+  <si>
+    <t>ISIC 27</t>
+  </si>
+  <si>
+    <t>ISIC 28</t>
+  </si>
+  <si>
+    <t>ISIC 29</t>
+  </si>
+  <si>
+    <t>ISIC 30</t>
+  </si>
+  <si>
+    <t>ISIC 31T33</t>
+  </si>
+  <si>
+    <t>ISIC 41T43</t>
+  </si>
+  <si>
+    <t>ISIC 45T47</t>
+  </si>
+  <si>
+    <t>ISIC 49T53</t>
+  </si>
+  <si>
+    <t>ISIC 55T56</t>
+  </si>
+  <si>
+    <t>ISIC 58T60</t>
+  </si>
+  <si>
+    <t>ISIC 61</t>
+  </si>
+  <si>
+    <t>ISIC 62T63</t>
+  </si>
+  <si>
+    <t>ISIC 64T66</t>
+  </si>
+  <si>
+    <t>ISIC 68</t>
+  </si>
+  <si>
+    <t>ISIC 69T82</t>
+  </si>
+  <si>
+    <t>ISIC 84</t>
+  </si>
+  <si>
+    <t>ISIC 85</t>
+  </si>
+  <si>
+    <t>ISIC 86T88</t>
+  </si>
+  <si>
+    <t>ISIC 90T96</t>
+  </si>
+  <si>
+    <t>Sources:</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>Unit: %</t>
+  </si>
+  <si>
+    <t>ISIC 20</t>
+  </si>
+  <si>
+    <t>ISIC 21</t>
+  </si>
+  <si>
+    <t>ISIC 05</t>
+  </si>
+  <si>
+    <t>ISIC 06</t>
+  </si>
+  <si>
+    <t>ISIC 231</t>
+  </si>
+  <si>
+    <t>ISIC 239</t>
+  </si>
+  <si>
+    <t>ISIC 241</t>
+  </si>
+  <si>
+    <t>ISIC 242</t>
+  </si>
+  <si>
+    <t>ISIC 351</t>
+  </si>
+  <si>
+    <t>ISIC 352T353</t>
+  </si>
+  <si>
+    <t>ISIC 36T39</t>
+  </si>
+  <si>
     <t>SoCTaSCbRIC Share of CCS Transportation and Storage Costs by Recipient ISIC Code</t>
   </si>
   <si>
-    <t>Sources:</t>
-  </si>
-  <si>
     <t>None needed</t>
-  </si>
-  <si>
-    <t>Notes:</t>
-  </si>
-  <si>
-    <t>Unit: %</t>
-  </si>
-  <si>
-    <t>ISIC 01T03</t>
-  </si>
-  <si>
-    <t>ISIC 05</t>
-  </si>
-  <si>
-    <t>ISIC 06</t>
-  </si>
-  <si>
-    <t>ISIC 07T08</t>
-  </si>
-  <si>
-    <t>ISIC 09</t>
-  </si>
-  <si>
-    <t>ISIC 10T12</t>
-  </si>
-  <si>
-    <t>ISIC 13T15</t>
-  </si>
-  <si>
-    <t>ISIC 16</t>
-  </si>
-  <si>
-    <t>ISIC 17T18</t>
-  </si>
-  <si>
-    <t>ISIC 19</t>
-  </si>
-  <si>
-    <t>ISIC 20</t>
-  </si>
-  <si>
-    <t>ISIC 21</t>
-  </si>
-  <si>
-    <t>ISIC 22</t>
-  </si>
-  <si>
-    <t>ISIC 231</t>
-  </si>
-  <si>
-    <t>ISIC 239</t>
-  </si>
-  <si>
-    <t>ISIC 241</t>
-  </si>
-  <si>
-    <t>ISIC 242</t>
-  </si>
-  <si>
-    <t>ISIC 25</t>
-  </si>
-  <si>
-    <t>ISIC 26</t>
-  </si>
-  <si>
-    <t>ISIC 27</t>
-  </si>
-  <si>
-    <t>ISIC 28</t>
-  </si>
-  <si>
-    <t>ISIC 29</t>
-  </si>
-  <si>
-    <t>ISIC 30</t>
-  </si>
-  <si>
-    <t>ISIC 31T33</t>
-  </si>
-  <si>
-    <t>ISIC 351</t>
-  </si>
-  <si>
-    <t>ISIC 352T353</t>
-  </si>
-  <si>
-    <t>ISIC 36T39</t>
-  </si>
-  <si>
-    <t>ISIC 41T43</t>
-  </si>
-  <si>
-    <t>ISIC 45T47</t>
-  </si>
-  <si>
-    <t>ISIC 49T53</t>
-  </si>
-  <si>
-    <t>ISIC 55T56</t>
-  </si>
-  <si>
-    <t>ISIC 58T60</t>
-  </si>
-  <si>
-    <t>ISIC 61</t>
-  </si>
-  <si>
-    <t>ISIC 62T63</t>
-  </si>
-  <si>
-    <t>ISIC 64T66</t>
-  </si>
-  <si>
-    <t>ISIC 68</t>
-  </si>
-  <si>
-    <t>ISIC 69T82</t>
-  </si>
-  <si>
-    <t>ISIC 84</t>
-  </si>
-  <si>
-    <t>ISIC 85</t>
-  </si>
-  <si>
-    <t>ISIC 86T88</t>
-  </si>
-  <si>
-    <t>ISIC 90T96</t>
-  </si>
-  <si>
-    <t>ISIC 97T98</t>
   </si>
   <si>
     <t>CCS transportation and storage costs</t>
@@ -187,7 +185,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -520,24 +518,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -551,146 +549,146 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AQ2"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.28515625" customWidth="1"/>
-    <col min="2" max="26" width="9.85546875" customWidth="1"/>
-    <col min="27" max="27" width="12.28515625" customWidth="1"/>
-    <col min="28" max="43" width="9.85546875" customWidth="1"/>
+    <col min="1" max="1" width="40.26953125" customWidth="1"/>
+    <col min="2" max="26" width="9.81640625" customWidth="1"/>
+    <col min="27" max="27" width="12.26953125" customWidth="1"/>
+    <col min="28" max="43" width="9.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="L1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="O1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AB1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AF1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AG1" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AK1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="AL1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="AM1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AN1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO1" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AP1" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="AQ1" s="2" t="s">
-        <v>46</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:43">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -825,175 +823,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
-    <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="79748b23-d81a-423e-9112-21109dc864e6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8EDCDEC6-0F4D-43C6-8953-76F174812A7D}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5218C100-F01B-4895-B2EF-E90DE9BA17C4}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B998777-0005-408F-AF3E-F91740D6DA17}"/>
 </file>
</xml_diff>